<commit_message>
Kedai Renjana: replace Indonesian screenshots with English ones and update README and model
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CsVrqfsAbWrWoYGEZaeovJ
</commit_message>
<xml_diff>
--- a/Excel-Kedai-Renjana-Budget-Cashflow-Planning/model/Kedai-Renjana-Budget-Model.xlsx
+++ b/Excel-Kedai-Renjana-Budget-Cashflow-Planning/model/Kedai-Renjana-Budget-Model.xlsx
@@ -21,7 +21,7 @@
     <sheet name="New_Outlet_Scenario" sheetId="7" r:id="rId6"/>
     <sheet name="Scenario Summary" sheetId="8" r:id="rId7"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
   <pivotCaches>
     <pivotCache cacheId="2" r:id="rId8"/>
     <pivotCache cacheId="3" r:id="rId9"/>
@@ -53546,7 +53546,7 @@
       </c>
       <c r="N27" s="63"/>
       <c r="O27" s="31">
-        <v>2.5988438045062239</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:17" ht="27" customHeight="1" x14ac:dyDescent="0.3">
@@ -53629,23 +53629,23 @@
       </c>
       <c r="G29" s="17">
         <f>P29+Q29</f>
-        <v>63488199.805922844</v>
+        <v>39054826.379705645</v>
       </c>
       <c r="H29" s="17">
         <f>D29-G29</f>
-        <v>-10981150.082521327</v>
+        <v>13452223.343695872</v>
       </c>
       <c r="I29" s="17">
         <f>I25+H29</f>
-        <v>221163849.91747868</v>
+        <v>245597223.34369588</v>
       </c>
       <c r="J29" s="17">
         <f>B29-P29</f>
-        <v>-5004535.2649606466</v>
+        <v>11498199.006360374</v>
       </c>
       <c r="K29" s="17">
         <f>C29-Q29</f>
-        <v>-5976614.8175606802</v>
+        <v>1954024.337335499</v>
       </c>
       <c r="L29" s="18">
         <f>B29*32.3%</f>
@@ -53665,11 +53665,11 @@
       </c>
       <c r="P29" s="18">
         <f>N29 + L29*(1-55%) + L29*55%*(1+$O$27)</f>
-        <v>40749141.440821052</v>
+        <v>24246407.16950003</v>
       </c>
       <c r="Q29" s="18">
         <f>O29 + M29*(1-55%) + M29*55%*(1+$O$27)</f>
-        <v>22739058.365101792</v>
+        <v>14808419.210205613</v>
       </c>
     </row>
     <row r="30" spans="1:17" x14ac:dyDescent="0.3">
@@ -53699,23 +53699,23 @@
       </c>
       <c r="G30" s="10">
         <f t="shared" ref="G30:G40" si="8">P30+Q30</f>
-        <v>65922072.747116849</v>
+        <v>40717435.307458445</v>
       </c>
       <c r="H30" s="10">
         <f t="shared" ref="H30:H40" si="9">D30-G30</f>
-        <v>-11867805.184674606</v>
+        <v>13336832.254983798</v>
       </c>
       <c r="I30" s="10">
         <f t="shared" ref="I30:I40" si="10">I29+H30</f>
-        <v>209296044.73280406</v>
+        <v>258934055.59867966</v>
       </c>
       <c r="J30" s="10">
         <f t="shared" ref="J30:J40" si="11">B30-P30</f>
-        <v>-6246007.3102269769</v>
+        <v>8672207.645919446</v>
       </c>
       <c r="K30" s="10">
         <f t="shared" ref="K30:K40" si="12">C30-Q30</f>
-        <v>-5621797.8744476251</v>
+        <v>4664624.6090643555</v>
       </c>
       <c r="L30" s="23">
         <f t="shared" ref="L30:L40" si="13">B30*32.3%</f>
@@ -53735,11 +53735,11 @@
       </c>
       <c r="P30" s="23">
         <f t="shared" ref="P30:P40" si="17">N30 + L30*(1-55%) + L30*55%*(1+$O$27)</f>
-        <v>38558575.01489976</v>
+        <v>23640360.058753338</v>
       </c>
       <c r="Q30" s="23">
         <f t="shared" ref="Q30:Q40" si="18">O30 + M30*(1-55%) + M30*55%*(1+$O$27)</f>
-        <v>27363497.732217088</v>
+        <v>17077075.248705108</v>
       </c>
     </row>
     <row r="31" spans="1:17" x14ac:dyDescent="0.3">
@@ -53769,23 +53769,23 @@
       </c>
       <c r="G31" s="17">
         <f t="shared" si="8"/>
-        <v>70466300.834242135</v>
+        <v>41951599.092411056</v>
       </c>
       <c r="H31" s="17">
         <f t="shared" si="9"/>
-        <v>-9339402.0326024443</v>
+        <v>19175299.709228635</v>
       </c>
       <c r="I31" s="17">
         <f t="shared" si="10"/>
-        <v>199956642.70020163</v>
+        <v>278109355.3079083</v>
       </c>
       <c r="J31" s="17">
         <f t="shared" si="11"/>
-        <v>-4783447.1470923722</v>
+        <v>11593740.912208669</v>
       </c>
       <c r="K31" s="17">
         <f t="shared" si="12"/>
-        <v>-4555954.8855100684</v>
+        <v>7581558.797019966</v>
       </c>
       <c r="L31" s="18">
         <f t="shared" si="13"/>
@@ -53805,11 +53805,11 @@
       </c>
       <c r="P31" s="18">
         <f t="shared" si="17"/>
-        <v>40256122.63366548</v>
+        <v>23878934.57436444</v>
       </c>
       <c r="Q31" s="18">
         <f t="shared" si="18"/>
-        <v>30210178.200576652</v>
+        <v>18072664.518046618</v>
       </c>
     </row>
     <row r="32" spans="1:17" x14ac:dyDescent="0.3">
@@ -53839,23 +53839,23 @@
       </c>
       <c r="G32" s="10">
         <f t="shared" si="8"/>
-        <v>69340397.687391937</v>
+        <v>41851226.72023864</v>
       </c>
       <c r="H32" s="10">
         <f t="shared" si="9"/>
-        <v>-10396277.778172314</v>
+        <v>17092893.18898098</v>
       </c>
       <c r="I32" s="10">
         <f t="shared" si="10"/>
-        <v>189560364.92202932</v>
+        <v>295202248.4968893</v>
       </c>
       <c r="J32" s="10">
         <f t="shared" si="11"/>
-        <v>-5397555.9336083457</v>
+        <v>10689557.316185325</v>
       </c>
       <c r="K32" s="10">
         <f t="shared" si="12"/>
-        <v>-4998721.8445639759</v>
+        <v>6403335.872795656</v>
       </c>
       <c r="L32" s="23">
         <f t="shared" si="13"/>
@@ -53875,11 +53875,11 @@
       </c>
       <c r="P32" s="23">
         <f t="shared" si="17"/>
-        <v>40241934.941736832</v>
+        <v>24154821.69194316</v>
       </c>
       <c r="Q32" s="23">
         <f t="shared" si="18"/>
-        <v>29098462.745655112</v>
+        <v>17696405.02829548</v>
       </c>
     </row>
     <row r="33" spans="1:17" x14ac:dyDescent="0.3">
@@ -53909,23 +53909,23 @@
       </c>
       <c r="G33" s="17">
         <f t="shared" si="8"/>
-        <v>74687386.668340042</v>
+        <v>45751939.34995618</v>
       </c>
       <c r="H33" s="17">
         <f t="shared" si="9"/>
-        <v>-12627491.460883781</v>
+        <v>16307955.857500084</v>
       </c>
       <c r="I33" s="17">
         <f t="shared" si="10"/>
-        <v>176932873.46114552</v>
+        <v>311510204.35438937</v>
       </c>
       <c r="J33" s="17">
         <f t="shared" si="11"/>
-        <v>-6166571.6695596501</v>
+        <v>11045298.055043206</v>
       </c>
       <c r="K33" s="17">
         <f t="shared" si="12"/>
-        <v>-6460919.7913241275</v>
+        <v>5262657.802456878</v>
       </c>
       <c r="L33" s="18">
         <f t="shared" si="13"/>
@@ -53945,11 +53945,11 @@
       </c>
       <c r="P33" s="18">
         <f t="shared" si="17"/>
-        <v>43447151.647467487</v>
+        <v>26235281.92286463</v>
       </c>
       <c r="Q33" s="18">
         <f t="shared" si="18"/>
-        <v>31240235.020872552</v>
+        <v>19516657.427091546</v>
       </c>
     </row>
     <row r="34" spans="1:17" x14ac:dyDescent="0.3">
@@ -53979,23 +53979,23 @@
       </c>
       <c r="G34" s="10">
         <f t="shared" si="8"/>
-        <v>71010797.803272605</v>
+        <v>42276369.99027063</v>
       </c>
       <c r="H34" s="10">
         <f t="shared" si="9"/>
-        <v>-9381005.4845878184</v>
+        <v>19353422.328414157</v>
       </c>
       <c r="I34" s="10">
         <f t="shared" si="10"/>
-        <v>167551867.9765577</v>
+        <v>330863626.6828035</v>
       </c>
       <c r="J34" s="10">
         <f t="shared" si="11"/>
-        <v>-4446644.8538789302</v>
+        <v>12665475.825557362</v>
       </c>
       <c r="K34" s="10">
         <f t="shared" si="12"/>
-        <v>-4934360.630708877</v>
+        <v>6687946.502856795</v>
       </c>
       <c r="L34" s="23">
         <f t="shared" si="13"/>
@@ -54015,11 +54015,11 @@
       </c>
       <c r="P34" s="23">
         <f t="shared" si="17"/>
-        <v>41511170.311531104</v>
+        <v>24399049.63209481</v>
       </c>
       <c r="Q34" s="23">
         <f t="shared" si="18"/>
-        <v>29499627.491741493</v>
+        <v>17877320.35817582</v>
       </c>
     </row>
     <row r="35" spans="1:17" x14ac:dyDescent="0.3">
@@ -54049,23 +54049,23 @@
       </c>
       <c r="G35" s="17">
         <f t="shared" si="8"/>
-        <v>65071868.416676939</v>
+        <v>40239549.89482429</v>
       </c>
       <c r="H35" s="17">
         <f t="shared" si="9"/>
-        <v>-11642307.768117458</v>
+        <v>13190010.753735192</v>
       </c>
       <c r="I35" s="17">
         <f t="shared" si="10"/>
-        <v>155909560.20844024</v>
+        <v>344053637.4365387</v>
       </c>
       <c r="J35" s="17">
         <f t="shared" si="11"/>
-        <v>-4591993.4609711766</v>
+        <v>13425321.139832944</v>
       </c>
       <c r="K35" s="17">
         <f t="shared" si="12"/>
-        <v>-7050314.3071462829</v>
+        <v>-235310.38609775528</v>
       </c>
       <c r="L35" s="18">
         <f t="shared" si="13"/>
@@ -54085,11 +54085,11 @@
       </c>
       <c r="P35" s="18">
         <f t="shared" si="17"/>
-        <v>43617151.605311215</v>
+        <v>25599837.004507095</v>
       </c>
       <c r="Q35" s="18">
         <f t="shared" si="18"/>
-        <v>21454716.811365724</v>
+        <v>14639712.890317196</v>
       </c>
     </row>
     <row r="36" spans="1:17" x14ac:dyDescent="0.3">
@@ -54119,23 +54119,23 @@
       </c>
       <c r="G36" s="10">
         <f t="shared" si="8"/>
-        <v>72652900.903434187</v>
+        <v>42840085.81094011</v>
       </c>
       <c r="H36" s="10">
         <f t="shared" si="9"/>
-        <v>-8721498.0178193748</v>
+        <v>21091317.074674703</v>
       </c>
       <c r="I36" s="10">
         <f t="shared" si="10"/>
-        <v>147188062.19062087</v>
+        <v>365144954.5112134</v>
       </c>
       <c r="J36" s="10">
         <f t="shared" si="11"/>
-        <v>-4185189.5676898435</v>
+        <v>13352871.00001517</v>
       </c>
       <c r="K36" s="10">
         <f t="shared" si="12"/>
-        <v>-4536308.4501295388</v>
+        <v>7738446.074659534</v>
       </c>
       <c r="L36" s="23">
         <f t="shared" si="13"/>
@@ -54155,11 +54155,11 @@
       </c>
       <c r="P36" s="23">
         <f t="shared" si="17"/>
-        <v>42172292.660686597</v>
+        <v>24634232.092981584</v>
       </c>
       <c r="Q36" s="23">
         <f t="shared" si="18"/>
-        <v>30480608.242747597</v>
+        <v>18205853.717958525</v>
       </c>
     </row>
     <row r="37" spans="1:17" x14ac:dyDescent="0.3">
@@ -54189,23 +54189,23 @@
       </c>
       <c r="G37" s="17">
         <f t="shared" si="8"/>
-        <v>74776322.17338717</v>
+        <v>44584838.25620708</v>
       </c>
       <c r="H37" s="17">
         <f t="shared" si="9"/>
-        <v>-10010911.186562255</v>
+        <v>20180572.730617836</v>
       </c>
       <c r="I37" s="17">
         <f t="shared" si="10"/>
-        <v>137177151.0040586</v>
+        <v>385325527.24183124</v>
       </c>
       <c r="J37" s="17">
         <f t="shared" si="11"/>
-        <v>-4038543.2583393455</v>
+        <v>14142153.399203125</v>
       </c>
       <c r="K37" s="17">
         <f t="shared" si="12"/>
-        <v>-5972367.9282229058</v>
+        <v>6038419.331414711</v>
       </c>
       <c r="L37" s="18">
         <f t="shared" si="13"/>
@@ -54225,11 +54225,11 @@
       </c>
       <c r="P37" s="18">
         <f t="shared" si="17"/>
-        <v>43417583.80654642</v>
+        <v>25236887.14900395</v>
       </c>
       <c r="Q37" s="18">
         <f t="shared" si="18"/>
-        <v>31358738.36684075</v>
+        <v>19347951.107203133</v>
       </c>
     </row>
     <row r="38" spans="1:17" x14ac:dyDescent="0.3">
@@ -54259,23 +54259,23 @@
       </c>
       <c r="G38" s="10">
         <f t="shared" si="8"/>
-        <v>73773016.999262765</v>
+        <v>42949299.454449356</v>
       </c>
       <c r="H38" s="10">
         <f t="shared" si="9"/>
-        <v>-7670067.0764600933</v>
+        <v>23153650.468353316</v>
       </c>
       <c r="I38" s="10">
         <f t="shared" si="10"/>
-        <v>129507083.92759851</v>
+        <v>408479177.7101846</v>
       </c>
       <c r="J38" s="10">
         <f t="shared" si="11"/>
-        <v>-3674193.8426270038</v>
+        <v>14530006.900270801</v>
       </c>
       <c r="K38" s="10">
         <f t="shared" si="12"/>
-        <v>-3995873.2338330932</v>
+        <v>8623643.568082515</v>
       </c>
       <c r="L38" s="23">
         <f t="shared" si="13"/>
@@ -54295,11 +54295,11 @@
       </c>
       <c r="P38" s="23">
         <f t="shared" si="17"/>
-        <v>43104143.789285123</v>
+        <v>24899943.04638732</v>
       </c>
       <c r="Q38" s="23">
         <f t="shared" si="18"/>
-        <v>30668873.209977642</v>
+        <v>18049356.408062033</v>
       </c>
     </row>
     <row r="39" spans="1:17" x14ac:dyDescent="0.3">
@@ -54329,23 +54329,23 @@
       </c>
       <c r="G39" s="17">
         <f t="shared" si="8"/>
-        <v>72950528.452385709</v>
+        <v>42843276.75298412</v>
       </c>
       <c r="H39" s="17">
         <f t="shared" si="9"/>
-        <v>-8393404.0632568896</v>
+        <v>21713847.636144698</v>
       </c>
       <c r="I39" s="17">
         <f t="shared" si="10"/>
-        <v>121113679.86434162</v>
+        <v>430193025.3463293</v>
       </c>
       <c r="J39" s="17">
         <f t="shared" si="11"/>
-        <v>-4766585.7827206105</v>
+        <v>12836254.33730521</v>
       </c>
       <c r="K39" s="17">
         <f t="shared" si="12"/>
-        <v>-3626818.2805362716</v>
+        <v>8877593.298839495</v>
       </c>
       <c r="L39" s="18">
         <f t="shared" si="13"/>
@@ -54365,11 +54365,11 @@
       </c>
       <c r="P39" s="18">
         <f t="shared" si="17"/>
-        <v>42894000.144619025</v>
+        <v>25291160.024593204</v>
       </c>
       <c r="Q39" s="18">
         <f t="shared" si="18"/>
-        <v>30056528.30776668</v>
+        <v>17552116.728390913</v>
       </c>
     </row>
     <row r="40" spans="1:17" x14ac:dyDescent="0.3">
@@ -54399,23 +54399,23 @@
       </c>
       <c r="G40" s="10">
         <f t="shared" si="8"/>
-        <v>84211875.21387665</v>
+        <v>48500340.86351147</v>
       </c>
       <c r="H40" s="10">
         <f t="shared" si="9"/>
-        <v>-7533537.8143417388</v>
+        <v>28177996.536023438</v>
       </c>
       <c r="I40" s="10">
         <f t="shared" si="10"/>
-        <v>113580142.04999988</v>
+        <v>458371021.8823527</v>
       </c>
       <c r="J40" s="10">
         <f t="shared" si="11"/>
-        <v>-2601996.8850251883</v>
+        <v>20269771.247218356</v>
       </c>
       <c r="K40" s="10">
         <f t="shared" si="12"/>
-        <v>-4931540.9293165579</v>
+        <v>7908225.288805079</v>
       </c>
       <c r="L40" s="23">
         <f t="shared" si="13"/>
@@ -54435,11 +54435,11 @@
       </c>
       <c r="P40" s="23">
         <f t="shared" si="17"/>
-        <v>52141808.348474063</v>
+        <v>29270040.21623052</v>
       </c>
       <c r="Q40" s="23">
         <f t="shared" si="18"/>
-        <v>32070066.865402587</v>
+        <v>19230300.64728095</v>
       </c>
     </row>
     <row r="41" spans="1:17" x14ac:dyDescent="0.3">
@@ -54481,11 +54481,11 @@
       <c r="A44" s="32"/>
       <c r="B44" s="33">
         <f>I40</f>
-        <v>113580142.04999988</v>
+        <v>458371021.8823527</v>
       </c>
       <c r="C44" s="33">
         <f>AVERAGE(H29:H40)</f>
-        <v>-9880404.829166675</v>
+        <v>18852168.49019606</v>
       </c>
       <c r="F44" s="15"/>
       <c r="G44" s="15"/>
@@ -54717,7 +54717,7 @@
       </c>
       <c r="M6" s="51">
         <f>Projection!I25+Projection!H29+L6</f>
-        <v>127538476.81747869</v>
+        <v>151971850.24369588</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.3">
@@ -54764,7 +54764,7 @@
       </c>
       <c r="M7" s="51">
         <f>M6+Projection!H30+L7</f>
-        <v>115715149.29280408</v>
+        <v>165353160.1586797</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.3">
@@ -54811,7 +54811,7 @@
       </c>
       <c r="M8" s="51">
         <f>M7+Projection!H31+L8</f>
-        <v>108229229.91020164</v>
+        <v>186381942.51790833</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.3">
@@ -54858,7 +54858,7 @@
       </c>
       <c r="M9" s="51">
         <f>M8+Projection!H32+L9</f>
-        <v>101495439.77202933</v>
+        <v>207137323.34688932</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.3">
@@ -54905,7 +54905,7 @@
       </c>
       <c r="M10" s="51">
         <f>M9+Projection!H33+L10</f>
-        <v>94200286.71114555</v>
+        <v>228777617.6043894</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.3">
@@ -54952,7 +54952,7 @@
       </c>
       <c r="M11" s="51">
         <f>M10+Projection!H34+L11</f>
-        <v>91543161.926557735</v>
+        <v>254854920.63280356</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.3">
@@ -54999,7 +54999,7 @@
       </c>
       <c r="M12" s="51">
         <f>M11+Projection!H35+L12</f>
-        <v>88016277.158440277</v>
+        <v>276160354.38653874</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.3">
@@ -55046,7 +55046,7 @@
       </c>
       <c r="M13" s="51">
         <f>M12+Projection!H36+L13</f>
-        <v>87410202.140620902</v>
+        <v>305367094.46121347</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.3">
@@ -55093,7 +55093,7 @@
       </c>
       <c r="M14" s="51">
         <f>M13+Projection!H37+L14</f>
-        <v>85514713.954058647</v>
+        <v>333663090.1918313</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.3">
@@ -55140,7 +55140,7 @@
       </c>
       <c r="M15" s="51">
         <f>M14+Projection!H38+L15</f>
-        <v>85960069.877598554</v>
+        <v>364932163.6601846</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.3">
@@ -55187,7 +55187,7 @@
       </c>
       <c r="M16" s="51">
         <f>M15+Projection!H39+L16</f>
-        <v>85682088.814341664</v>
+        <v>394761434.2963293</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.3">
@@ -55234,7 +55234,7 @@
       </c>
       <c r="M17" s="51">
         <f>M16+Projection!H40+L17</f>
-        <v>86263973.999999925</v>
+        <v>431054853.83235276</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.3">

</xml_diff>